<commit_message>
APR: lista de presença em todas as APRs e remoção de redundâncias
- Molde ganha a página 'LISTA DE PRESENÇA DO TREINAMENTO DA APR', gerada
  sempre como última página, com datas, descrição, responsáveis e local.
- Textos padrão revisados: linhas repetidas unificadas (planejamento,
  transporte, rota de fuga, bloqueio, 5S).
- Catálogo com temas por medida e temas cobertos por etapa: o gerador
  omite o que as etapas padrão ou outros riscos já disseram e lista o que
  omitiu. Novo risco nh3_proximidade e verificador de redundância.
- modelo-para-skill: lições registradas (ver o exemplo até a última página
  e evitar redundância entre seções).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNFTn9Bz7Q4cwJtHtFiNDd
</commit_message>
<xml_diff>
--- a/.claude/skills/apr-seguranca/assets/modelo-anexo9.xlsx
+++ b/.claude/skills/apr-seguranca/assets/modelo-anexo9.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APR Execução(Modelo) " sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'APR Execução(Modelo) '!$A$1:$R$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'APR Execução(Modelo) '!$A$1:$R$46</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -840,7 +840,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="285">
+  <cellXfs count="298">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -1632,6 +1632,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2033,7 +2066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:T19"/>
+  <dimension ref="A2:T46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col width="5.28515625" customWidth="1" style="1" min="1" max="1"/>
@@ -2560,33 +2593,697 @@
       <c r="Q19" s="21" t="n"/>
       <c r="R19" s="21" t="n"/>
     </row>
-    <row r="20" ht="21" customHeight="1"/>
-    <row r="21" ht="21" customHeight="1"/>
-    <row r="22" ht="17.1" customHeight="1"/>
-    <row r="23" ht="30" customHeight="1"/>
-    <row r="24" ht="28.9" customHeight="1"/>
-    <row r="25" ht="26.45" customHeight="1"/>
-    <row r="26" ht="33" customHeight="1"/>
-    <row r="27" ht="18" customHeight="1"/>
-    <row r="28" ht="17.1" customHeight="1"/>
-    <row r="29" ht="17.1" customHeight="1"/>
-    <row r="30" ht="48.6" customHeight="1"/>
-    <row r="31" ht="129.75" customHeight="1"/>
-    <row r="32" ht="164.25" customHeight="1"/>
-    <row r="33" ht="286.5" customHeight="1"/>
-    <row r="34" ht="30" customHeight="1"/>
-    <row r="35" ht="35.25" customHeight="1"/>
-    <row r="36" ht="28.5" customHeight="1"/>
-    <row r="37" ht="24.75" customHeight="1"/>
-    <row r="38" ht="24" customHeight="1" thickBot="1"/>
-    <row r="39" ht="21" customHeight="1"/>
-    <row r="40" ht="21" customHeight="1"/>
-    <row r="41" ht="17.1" customHeight="1"/>
-    <row r="42" ht="30" customHeight="1"/>
-    <row r="43" ht="28.9" customHeight="1"/>
-    <row r="44" ht="26.45" customHeight="1"/>
-    <row r="45" ht="33" customHeight="1"/>
-    <row r="46" ht="18" customHeight="1"/>
+    <row r="20" ht="51" customHeight="1">
+      <c r="B20" s="285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TJ MONTAGENS </t>
+        </is>
+      </c>
+      <c r="E20" s="253" t="n"/>
+      <c r="F20" s="214" t="inlineStr">
+        <is>
+          <t>ANEXO 9 - LISTA DE PRESENÇA DO TREINAMENTO DA APR / DECLARAÇÃO DE MÉTODO</t>
+        </is>
+      </c>
+      <c r="S20" s="22" t="n"/>
+      <c r="T20" s="23" t="n"/>
+    </row>
+    <row r="21" hidden="1" ht="408.75" customHeight="1">
+      <c r="B21" s="252" t="n"/>
+      <c r="E21" s="253" t="n"/>
+      <c r="F21" s="286" t="n"/>
+      <c r="G21" s="264" t="n"/>
+      <c r="H21" s="264" t="n"/>
+      <c r="I21" s="264" t="n"/>
+      <c r="J21" s="264" t="n"/>
+      <c r="K21" s="264" t="n"/>
+      <c r="L21" s="264" t="n"/>
+      <c r="M21" s="264" t="n"/>
+      <c r="N21" s="264" t="n"/>
+      <c r="O21" s="264" t="n"/>
+      <c r="P21" s="264" t="n"/>
+      <c r="Q21" s="264" t="n"/>
+      <c r="R21" s="264" t="n"/>
+      <c r="S21" s="24" t="n"/>
+      <c r="T21" s="25" t="n"/>
+    </row>
+    <row r="22" ht="25.5" customHeight="1">
+      <c r="B22" s="286" t="n"/>
+      <c r="C22" s="264" t="n"/>
+      <c r="D22" s="264" t="n"/>
+      <c r="E22" s="265" t="n"/>
+      <c r="F22" s="97" t="inlineStr">
+        <is>
+          <t>DATA PREVISTA DE INÍCIO:</t>
+        </is>
+      </c>
+      <c r="G22" s="256" t="n"/>
+      <c r="H22" s="26" t="n"/>
+      <c r="I22" s="97" t="inlineStr">
+        <is>
+          <t>DATA PREVISTA DE TÉRMINO:</t>
+        </is>
+      </c>
+      <c r="J22" s="255" t="n"/>
+      <c r="K22" s="255" t="n"/>
+      <c r="L22" s="255" t="n"/>
+      <c r="M22" s="255" t="n"/>
+      <c r="N22" s="256" t="n"/>
+      <c r="O22" s="26" t="n"/>
+      <c r="P22" s="255" t="n"/>
+      <c r="Q22" s="255" t="n"/>
+      <c r="R22" s="256" t="n"/>
+      <c r="S22" s="27" t="n"/>
+      <c r="T22" s="28" t="n"/>
+    </row>
+    <row r="23" ht="25.5" customHeight="1">
+      <c r="B23" s="99" t="inlineStr">
+        <is>
+          <t>DESCRIÇÃO DOS TRABALHOS:</t>
+        </is>
+      </c>
+      <c r="C23" s="255" t="n"/>
+      <c r="D23" s="255" t="n"/>
+      <c r="E23" s="256" t="n"/>
+      <c r="F23" s="146" t="n"/>
+      <c r="G23" s="255" t="n"/>
+      <c r="H23" s="255" t="n"/>
+      <c r="I23" s="255" t="n"/>
+      <c r="J23" s="255" t="n"/>
+      <c r="K23" s="255" t="n"/>
+      <c r="L23" s="255" t="n"/>
+      <c r="M23" s="255" t="n"/>
+      <c r="N23" s="255" t="n"/>
+      <c r="O23" s="255" t="n"/>
+      <c r="P23" s="255" t="n"/>
+      <c r="Q23" s="255" t="n"/>
+      <c r="R23" s="255" t="n"/>
+      <c r="S23" s="255" t="n"/>
+      <c r="T23" s="256" t="n"/>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="B24" s="99" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL DA EMPRESA:</t>
+        </is>
+      </c>
+      <c r="C24" s="255" t="n"/>
+      <c r="D24" s="255" t="n"/>
+      <c r="E24" s="256" t="n"/>
+      <c r="F24" s="147" t="n"/>
+      <c r="G24" s="255" t="n"/>
+      <c r="H24" s="255" t="n"/>
+      <c r="I24" s="255" t="n"/>
+      <c r="J24" s="255" t="n"/>
+      <c r="K24" s="255" t="n"/>
+      <c r="L24" s="255" t="n"/>
+      <c r="M24" s="256" t="n"/>
+      <c r="N24" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TELEFONE: </t>
+        </is>
+      </c>
+      <c r="O24" s="256" t="n"/>
+      <c r="P24" s="98" t="n"/>
+      <c r="Q24" s="255" t="n"/>
+      <c r="R24" s="255" t="n"/>
+      <c r="S24" s="255" t="n"/>
+      <c r="T24" s="256" t="n"/>
+    </row>
+    <row r="25" ht="23.25" customHeight="1">
+      <c r="B25" s="99" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL SEGURANÇA DA EMPRESA:</t>
+        </is>
+      </c>
+      <c r="C25" s="255" t="n"/>
+      <c r="D25" s="255" t="n"/>
+      <c r="E25" s="256" t="n"/>
+      <c r="F25" s="205" t="n"/>
+      <c r="G25" s="255" t="n"/>
+      <c r="H25" s="255" t="n"/>
+      <c r="I25" s="255" t="n"/>
+      <c r="J25" s="255" t="n"/>
+      <c r="K25" s="255" t="n"/>
+      <c r="L25" s="255" t="n"/>
+      <c r="M25" s="256" t="n"/>
+      <c r="N25" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TELEFONE: </t>
+        </is>
+      </c>
+      <c r="O25" s="256" t="n"/>
+      <c r="P25" s="98" t="n"/>
+      <c r="Q25" s="255" t="n"/>
+      <c r="R25" s="255" t="n"/>
+      <c r="S25" s="255" t="n"/>
+      <c r="T25" s="256" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="99" t="inlineStr">
+        <is>
+          <t>LOCAL DA ATIVIDADE:</t>
+        </is>
+      </c>
+      <c r="C26" s="255" t="n"/>
+      <c r="D26" s="255" t="n"/>
+      <c r="E26" s="256" t="n"/>
+      <c r="F26" s="147" t="n"/>
+      <c r="G26" s="255" t="n"/>
+      <c r="H26" s="255" t="n"/>
+      <c r="I26" s="255" t="n"/>
+      <c r="J26" s="255" t="n"/>
+      <c r="K26" s="255" t="n"/>
+      <c r="L26" s="255" t="n"/>
+      <c r="M26" s="255" t="n"/>
+      <c r="N26" s="255" t="n"/>
+      <c r="O26" s="255" t="n"/>
+      <c r="P26" s="255" t="n"/>
+      <c r="Q26" s="255" t="n"/>
+      <c r="R26" s="255" t="n"/>
+      <c r="S26" s="255" t="n"/>
+      <c r="T26" s="256" t="n"/>
+    </row>
+    <row r="27" ht="34.9" customHeight="1">
+      <c r="B27" s="204" t="inlineStr">
+        <is>
+          <t>Declaro que fui treinado e que estou ciente dos riscos e exposições inerentes as atividades que irei executar conforme esta APR / DECLARAÇÃO DE MÉTODOS especificados neste documento.</t>
+        </is>
+      </c>
+      <c r="C27" s="255" t="n"/>
+      <c r="D27" s="255" t="n"/>
+      <c r="E27" s="255" t="n"/>
+      <c r="F27" s="255" t="n"/>
+      <c r="G27" s="255" t="n"/>
+      <c r="H27" s="255" t="n"/>
+      <c r="I27" s="255" t="n"/>
+      <c r="J27" s="255" t="n"/>
+      <c r="K27" s="255" t="n"/>
+      <c r="L27" s="255" t="n"/>
+      <c r="M27" s="255" t="n"/>
+      <c r="N27" s="255" t="n"/>
+      <c r="O27" s="255" t="n"/>
+      <c r="P27" s="255" t="n"/>
+      <c r="Q27" s="255" t="n"/>
+      <c r="R27" s="255" t="n"/>
+      <c r="S27" s="255" t="n"/>
+      <c r="T27" s="256" t="n"/>
+    </row>
+    <row r="28" ht="16.5" customHeight="1">
+      <c r="B28" s="145" t="inlineStr">
+        <is>
+          <t>NOME</t>
+        </is>
+      </c>
+      <c r="C28" s="255" t="n"/>
+      <c r="D28" s="255" t="n"/>
+      <c r="E28" s="256" t="n"/>
+      <c r="F28" s="145" t="inlineStr">
+        <is>
+          <t>CARGO</t>
+        </is>
+      </c>
+      <c r="G28" s="255" t="n"/>
+      <c r="H28" s="256" t="n"/>
+      <c r="I28" s="145" t="inlineStr">
+        <is>
+          <t>ASSINATURA</t>
+        </is>
+      </c>
+      <c r="J28" s="255" t="n"/>
+      <c r="K28" s="255" t="n"/>
+      <c r="L28" s="255" t="n"/>
+      <c r="M28" s="255" t="n"/>
+      <c r="N28" s="255" t="n"/>
+      <c r="O28" s="255" t="n"/>
+      <c r="P28" s="256" t="n"/>
+      <c r="Q28" s="145" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="R28" s="256" t="n"/>
+      <c r="S28" s="145" t="n"/>
+      <c r="T28" s="256" t="n"/>
+    </row>
+    <row r="29" ht="40.15" customHeight="1">
+      <c r="B29" s="144" t="n"/>
+      <c r="C29" s="255" t="n"/>
+      <c r="D29" s="255" t="n"/>
+      <c r="E29" s="256" t="n"/>
+      <c r="F29" s="144" t="n"/>
+      <c r="G29" s="255" t="n"/>
+      <c r="H29" s="256" t="n"/>
+      <c r="I29" s="144" t="n"/>
+      <c r="J29" s="255" t="n"/>
+      <c r="K29" s="255" t="n"/>
+      <c r="L29" s="255" t="n"/>
+      <c r="M29" s="255" t="n"/>
+      <c r="N29" s="255" t="n"/>
+      <c r="O29" s="255" t="n"/>
+      <c r="P29" s="256" t="n"/>
+      <c r="Q29" s="144" t="n"/>
+      <c r="R29" s="256" t="n"/>
+      <c r="S29" s="144" t="n"/>
+      <c r="T29" s="256" t="n"/>
+    </row>
+    <row r="30" ht="40.15" customHeight="1">
+      <c r="B30" s="144" t="n"/>
+      <c r="C30" s="255" t="n"/>
+      <c r="D30" s="255" t="n"/>
+      <c r="E30" s="256" t="n"/>
+      <c r="F30" s="144" t="n"/>
+      <c r="G30" s="255" t="n"/>
+      <c r="H30" s="256" t="n"/>
+      <c r="I30" s="144" t="n"/>
+      <c r="J30" s="255" t="n"/>
+      <c r="K30" s="255" t="n"/>
+      <c r="L30" s="255" t="n"/>
+      <c r="M30" s="255" t="n"/>
+      <c r="N30" s="255" t="n"/>
+      <c r="O30" s="255" t="n"/>
+      <c r="P30" s="256" t="n"/>
+      <c r="Q30" s="144" t="n"/>
+      <c r="R30" s="256" t="n"/>
+      <c r="S30" s="144" t="n"/>
+      <c r="T30" s="256" t="n"/>
+    </row>
+    <row r="31" ht="40.15" customHeight="1">
+      <c r="B31" s="144" t="n"/>
+      <c r="C31" s="255" t="n"/>
+      <c r="D31" s="255" t="n"/>
+      <c r="E31" s="256" t="n"/>
+      <c r="F31" s="144" t="n"/>
+      <c r="G31" s="255" t="n"/>
+      <c r="H31" s="256" t="n"/>
+      <c r="I31" s="144" t="n"/>
+      <c r="J31" s="255" t="n"/>
+      <c r="K31" s="255" t="n"/>
+      <c r="L31" s="255" t="n"/>
+      <c r="M31" s="255" t="n"/>
+      <c r="N31" s="255" t="n"/>
+      <c r="O31" s="255" t="n"/>
+      <c r="P31" s="256" t="n"/>
+      <c r="Q31" s="144" t="n"/>
+      <c r="R31" s="256" t="n"/>
+      <c r="S31" s="144" t="n"/>
+      <c r="T31" s="256" t="n"/>
+    </row>
+    <row r="32" ht="40.15" customHeight="1">
+      <c r="B32" s="144" t="n"/>
+      <c r="C32" s="255" t="n"/>
+      <c r="D32" s="255" t="n"/>
+      <c r="E32" s="256" t="n"/>
+      <c r="F32" s="144" t="n"/>
+      <c r="G32" s="255" t="n"/>
+      <c r="H32" s="256" t="n"/>
+      <c r="I32" s="144" t="n"/>
+      <c r="J32" s="255" t="n"/>
+      <c r="K32" s="255" t="n"/>
+      <c r="L32" s="255" t="n"/>
+      <c r="M32" s="255" t="n"/>
+      <c r="N32" s="255" t="n"/>
+      <c r="O32" s="255" t="n"/>
+      <c r="P32" s="256" t="n"/>
+      <c r="Q32" s="144" t="n"/>
+      <c r="R32" s="256" t="n"/>
+      <c r="S32" s="144" t="n"/>
+      <c r="T32" s="256" t="n"/>
+    </row>
+    <row r="33" ht="40.15" customHeight="1">
+      <c r="B33" s="144" t="n"/>
+      <c r="C33" s="255" t="n"/>
+      <c r="D33" s="255" t="n"/>
+      <c r="E33" s="256" t="n"/>
+      <c r="F33" s="144" t="n"/>
+      <c r="G33" s="255" t="n"/>
+      <c r="H33" s="256" t="n"/>
+      <c r="I33" s="144" t="n"/>
+      <c r="J33" s="255" t="n"/>
+      <c r="K33" s="255" t="n"/>
+      <c r="L33" s="255" t="n"/>
+      <c r="M33" s="255" t="n"/>
+      <c r="N33" s="255" t="n"/>
+      <c r="O33" s="255" t="n"/>
+      <c r="P33" s="256" t="n"/>
+      <c r="Q33" s="144" t="n"/>
+      <c r="R33" s="256" t="n"/>
+      <c r="S33" s="144" t="n"/>
+      <c r="T33" s="256" t="n"/>
+    </row>
+    <row r="34" ht="40.15" customHeight="1">
+      <c r="B34" s="144" t="n"/>
+      <c r="C34" s="255" t="n"/>
+      <c r="D34" s="255" t="n"/>
+      <c r="E34" s="256" t="n"/>
+      <c r="F34" s="144" t="n"/>
+      <c r="G34" s="255" t="n"/>
+      <c r="H34" s="256" t="n"/>
+      <c r="I34" s="144" t="n"/>
+      <c r="J34" s="255" t="n"/>
+      <c r="K34" s="255" t="n"/>
+      <c r="L34" s="255" t="n"/>
+      <c r="M34" s="255" t="n"/>
+      <c r="N34" s="255" t="n"/>
+      <c r="O34" s="255" t="n"/>
+      <c r="P34" s="256" t="n"/>
+      <c r="Q34" s="144" t="n"/>
+      <c r="R34" s="256" t="n"/>
+      <c r="S34" s="144" t="n"/>
+      <c r="T34" s="256" t="n"/>
+    </row>
+    <row r="35" ht="40.15" customHeight="1">
+      <c r="B35" s="144" t="n"/>
+      <c r="C35" s="255" t="n"/>
+      <c r="D35" s="255" t="n"/>
+      <c r="E35" s="256" t="n"/>
+      <c r="F35" s="144" t="n"/>
+      <c r="G35" s="255" t="n"/>
+      <c r="H35" s="256" t="n"/>
+      <c r="I35" s="144" t="n"/>
+      <c r="J35" s="255" t="n"/>
+      <c r="K35" s="255" t="n"/>
+      <c r="L35" s="255" t="n"/>
+      <c r="M35" s="255" t="n"/>
+      <c r="N35" s="255" t="n"/>
+      <c r="O35" s="255" t="n"/>
+      <c r="P35" s="256" t="n"/>
+      <c r="Q35" s="144" t="n"/>
+      <c r="R35" s="256" t="n"/>
+      <c r="S35" s="144" t="n"/>
+      <c r="T35" s="256" t="n"/>
+    </row>
+    <row r="36" ht="40.15" customHeight="1">
+      <c r="B36" s="144" t="n"/>
+      <c r="C36" s="255" t="n"/>
+      <c r="D36" s="255" t="n"/>
+      <c r="E36" s="256" t="n"/>
+      <c r="F36" s="144" t="n"/>
+      <c r="G36" s="255" t="n"/>
+      <c r="H36" s="256" t="n"/>
+      <c r="I36" s="144" t="n"/>
+      <c r="J36" s="255" t="n"/>
+      <c r="K36" s="255" t="n"/>
+      <c r="L36" s="255" t="n"/>
+      <c r="M36" s="255" t="n"/>
+      <c r="N36" s="255" t="n"/>
+      <c r="O36" s="255" t="n"/>
+      <c r="P36" s="256" t="n"/>
+      <c r="Q36" s="144" t="n"/>
+      <c r="R36" s="256" t="n"/>
+      <c r="S36" s="144" t="n"/>
+      <c r="T36" s="144" t="n"/>
+    </row>
+    <row r="37" ht="40.15" customHeight="1">
+      <c r="B37" s="144" t="n"/>
+      <c r="C37" s="255" t="n"/>
+      <c r="D37" s="255" t="n"/>
+      <c r="E37" s="256" t="n"/>
+      <c r="F37" s="144" t="n"/>
+      <c r="G37" s="255" t="n"/>
+      <c r="H37" s="256" t="n"/>
+      <c r="I37" s="144" t="n"/>
+      <c r="J37" s="255" t="n"/>
+      <c r="K37" s="255" t="n"/>
+      <c r="L37" s="255" t="n"/>
+      <c r="M37" s="255" t="n"/>
+      <c r="N37" s="255" t="n"/>
+      <c r="O37" s="255" t="n"/>
+      <c r="P37" s="256" t="n"/>
+      <c r="Q37" s="144" t="n"/>
+      <c r="R37" s="256" t="n"/>
+      <c r="S37" s="144" t="n"/>
+      <c r="T37" s="144" t="n"/>
+    </row>
+    <row r="38" ht="40.15" customHeight="1" thickBot="1">
+      <c r="B38" s="144" t="n"/>
+      <c r="C38" s="255" t="n"/>
+      <c r="D38" s="255" t="n"/>
+      <c r="E38" s="256" t="n"/>
+      <c r="F38" s="144" t="n"/>
+      <c r="G38" s="255" t="n"/>
+      <c r="H38" s="256" t="n"/>
+      <c r="I38" s="144" t="n"/>
+      <c r="J38" s="255" t="n"/>
+      <c r="K38" s="255" t="n"/>
+      <c r="L38" s="255" t="n"/>
+      <c r="M38" s="255" t="n"/>
+      <c r="N38" s="255" t="n"/>
+      <c r="O38" s="255" t="n"/>
+      <c r="P38" s="256" t="n"/>
+      <c r="Q38" s="144" t="n"/>
+      <c r="R38" s="256" t="n"/>
+      <c r="S38" s="144" t="n"/>
+      <c r="T38" s="144" t="n"/>
+    </row>
+    <row r="39" ht="40.15" customHeight="1">
+      <c r="B39" s="144" t="n"/>
+      <c r="C39" s="255" t="n"/>
+      <c r="D39" s="255" t="n"/>
+      <c r="E39" s="256" t="n"/>
+      <c r="F39" s="144" t="n"/>
+      <c r="G39" s="255" t="n"/>
+      <c r="H39" s="256" t="n"/>
+      <c r="I39" s="144" t="n"/>
+      <c r="J39" s="255" t="n"/>
+      <c r="K39" s="255" t="n"/>
+      <c r="L39" s="255" t="n"/>
+      <c r="M39" s="255" t="n"/>
+      <c r="N39" s="255" t="n"/>
+      <c r="O39" s="255" t="n"/>
+      <c r="P39" s="256" t="n"/>
+      <c r="Q39" s="144" t="n"/>
+      <c r="R39" s="256" t="n"/>
+      <c r="S39" s="144" t="n"/>
+      <c r="T39" s="144" t="n"/>
+    </row>
+    <row r="40" ht="40.15" customHeight="1">
+      <c r="B40" s="144" t="n"/>
+      <c r="C40" s="255" t="n"/>
+      <c r="D40" s="255" t="n"/>
+      <c r="E40" s="256" t="n"/>
+      <c r="F40" s="144" t="n"/>
+      <c r="G40" s="255" t="n"/>
+      <c r="H40" s="256" t="n"/>
+      <c r="I40" s="144" t="n"/>
+      <c r="J40" s="255" t="n"/>
+      <c r="K40" s="255" t="n"/>
+      <c r="L40" s="255" t="n"/>
+      <c r="M40" s="255" t="n"/>
+      <c r="N40" s="255" t="n"/>
+      <c r="O40" s="255" t="n"/>
+      <c r="P40" s="256" t="n"/>
+      <c r="Q40" s="144" t="n"/>
+      <c r="R40" s="256" t="n"/>
+      <c r="S40" s="144" t="n"/>
+      <c r="T40" s="144" t="n"/>
+    </row>
+    <row r="41" ht="40.15" customHeight="1">
+      <c r="B41" s="144" t="n"/>
+      <c r="C41" s="255" t="n"/>
+      <c r="D41" s="255" t="n"/>
+      <c r="E41" s="256" t="n"/>
+      <c r="F41" s="144" t="n"/>
+      <c r="G41" s="255" t="n"/>
+      <c r="H41" s="256" t="n"/>
+      <c r="I41" s="144" t="n"/>
+      <c r="J41" s="255" t="n"/>
+      <c r="K41" s="255" t="n"/>
+      <c r="L41" s="255" t="n"/>
+      <c r="M41" s="255" t="n"/>
+      <c r="N41" s="255" t="n"/>
+      <c r="O41" s="255" t="n"/>
+      <c r="P41" s="256" t="n"/>
+      <c r="Q41" s="144" t="n"/>
+      <c r="R41" s="256" t="n"/>
+      <c r="S41" s="144" t="n"/>
+      <c r="T41" s="144" t="n"/>
+    </row>
+    <row r="42" ht="63.75" customHeight="1">
+      <c r="B42" s="287" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL DA EMPRESA:</t>
+        </is>
+      </c>
+      <c r="C42" s="282" t="n"/>
+      <c r="D42" s="282" t="n"/>
+      <c r="E42" s="282" t="n"/>
+      <c r="F42" s="288" t="n"/>
+      <c r="G42" s="197" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL - SEGURANÇA DO TRABALHO EMPRESA</t>
+        </is>
+      </c>
+      <c r="H42" s="256" t="n"/>
+      <c r="I42" s="197" t="inlineStr">
+        <is>
+          <t>SEGURANÇA DO TRABALHO AMBEV</t>
+        </is>
+      </c>
+      <c r="J42" s="255" t="n"/>
+      <c r="K42" s="255" t="n"/>
+      <c r="L42" s="255" t="n"/>
+      <c r="M42" s="255" t="n"/>
+      <c r="N42" s="256" t="n"/>
+      <c r="O42" s="289" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL AMBEV PELA ATIVIDADE</t>
+        </is>
+      </c>
+      <c r="P42" s="282" t="n"/>
+      <c r="Q42" s="282" t="n"/>
+      <c r="R42" s="283" t="n"/>
+      <c r="S42" s="33" t="n"/>
+      <c r="T42" s="33" t="n"/>
+    </row>
+    <row r="43" ht="37.15" customHeight="1">
+      <c r="B43" s="290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="C43" s="259" t="n"/>
+      <c r="D43" s="259" t="n"/>
+      <c r="E43" s="259" t="n"/>
+      <c r="F43" s="260" t="n"/>
+      <c r="G43" s="291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="H43" s="260" t="n"/>
+      <c r="I43" s="291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="J43" s="259" t="n"/>
+      <c r="K43" s="259" t="n"/>
+      <c r="L43" s="259" t="n"/>
+      <c r="M43" s="259" t="n"/>
+      <c r="N43" s="260" t="n"/>
+      <c r="O43" s="292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="P43" s="259" t="n"/>
+      <c r="Q43" s="259" t="n"/>
+      <c r="R43" s="259" t="n"/>
+      <c r="S43" s="259" t="n"/>
+      <c r="T43" s="293" t="n"/>
+    </row>
+    <row r="44" ht="38.65" customHeight="1">
+      <c r="B44" s="294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="C44" s="259" t="n"/>
+      <c r="D44" s="259" t="n"/>
+      <c r="E44" s="259" t="n"/>
+      <c r="F44" s="260" t="n"/>
+      <c r="G44" s="295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="H44" s="260" t="n"/>
+      <c r="I44" s="189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="J44" s="255" t="n"/>
+      <c r="K44" s="255" t="n"/>
+      <c r="L44" s="255" t="n"/>
+      <c r="M44" s="255" t="n"/>
+      <c r="N44" s="256" t="n"/>
+      <c r="O44" s="189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº do documento: </t>
+        </is>
+      </c>
+      <c r="P44" s="255" t="n"/>
+      <c r="Q44" s="255" t="n"/>
+      <c r="R44" s="255" t="n"/>
+      <c r="S44" s="255" t="n"/>
+      <c r="T44" s="256" t="n"/>
+    </row>
+    <row r="45" ht="25.5" customHeight="1">
+      <c r="B45" s="294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="C45" s="259" t="n"/>
+      <c r="D45" s="259" t="n"/>
+      <c r="E45" s="259" t="n"/>
+      <c r="F45" s="260" t="n"/>
+      <c r="G45" s="295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="H45" s="260" t="n"/>
+      <c r="I45" s="296" t="inlineStr">
+        <is>
+          <t>Contato:</t>
+        </is>
+      </c>
+      <c r="J45" s="259" t="n"/>
+      <c r="K45" s="259" t="n"/>
+      <c r="L45" s="259" t="n"/>
+      <c r="M45" s="259" t="n"/>
+      <c r="N45" s="260" t="n"/>
+      <c r="O45" s="292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="P45" s="259" t="n"/>
+      <c r="Q45" s="259" t="n"/>
+      <c r="R45" s="259" t="n"/>
+      <c r="S45" s="259" t="n"/>
+      <c r="T45" s="293" t="n"/>
+    </row>
+    <row r="46" ht="42" customHeight="1">
+      <c r="B46" s="297" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="C46" s="259" t="n"/>
+      <c r="D46" s="259" t="n"/>
+      <c r="E46" s="259" t="n"/>
+      <c r="F46" s="260" t="n"/>
+      <c r="G46" s="186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assinatura:                                                       </t>
+        </is>
+      </c>
+      <c r="H46" s="256" t="n"/>
+      <c r="I46" s="186" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="J46" s="255" t="n"/>
+      <c r="K46" s="255" t="n"/>
+      <c r="L46" s="255" t="n"/>
+      <c r="M46" s="255" t="n"/>
+      <c r="N46" s="256" t="n"/>
+      <c r="O46" s="186" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="P46" s="255" t="n"/>
+      <c r="Q46" s="255" t="n"/>
+      <c r="R46" s="255" t="n"/>
+      <c r="S46" s="255" t="n"/>
+      <c r="T46" s="256" t="n"/>
+    </row>
     <row r="47" ht="17.1" customHeight="1"/>
     <row r="48" ht="17.1" customHeight="1"/>
     <row r="49" ht="48.6" customHeight="1"/>
@@ -2771,51 +3468,153 @@
     <row r="228" ht="25.5" customHeight="1"/>
     <row r="229" ht="42" customHeight="1"/>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="146">
+    <mergeCell ref="I34:P34"/>
     <mergeCell ref="F18:H18"/>
+    <mergeCell ref="I22:N22"/>
     <mergeCell ref="I4:L4"/>
     <mergeCell ref="F17:H17"/>
+    <mergeCell ref="I36:P36"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="F41:H41"/>
+    <mergeCell ref="F25:M25"/>
+    <mergeCell ref="Q37:R37"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F23:T23"/>
+    <mergeCell ref="Q38:R38"/>
+    <mergeCell ref="Q40:R40"/>
     <mergeCell ref="B18:E18"/>
+    <mergeCell ref="S33:T33"/>
+    <mergeCell ref="I39:P39"/>
+    <mergeCell ref="I46:N46"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="O45:T45"/>
     <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B24:E24"/>
     <mergeCell ref="M7:R7"/>
+    <mergeCell ref="I43:N43"/>
+    <mergeCell ref="F38:H38"/>
+    <mergeCell ref="S28:T28"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="I9:O12"/>
+    <mergeCell ref="Q41:R41"/>
+    <mergeCell ref="O46:T46"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="Q36:R36"/>
     <mergeCell ref="I3:L3"/>
+    <mergeCell ref="S29:T29"/>
+    <mergeCell ref="S31:T31"/>
     <mergeCell ref="O14:R14"/>
     <mergeCell ref="H9:H12"/>
+    <mergeCell ref="F20:R21"/>
     <mergeCell ref="I14:N14"/>
+    <mergeCell ref="I28:P28"/>
     <mergeCell ref="F14:H14"/>
     <mergeCell ref="B2:E4"/>
     <mergeCell ref="G9:G12"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="F26:T26"/>
+    <mergeCell ref="Q39:R39"/>
     <mergeCell ref="F7:J7"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B35:E35"/>
     <mergeCell ref="F5:R5"/>
     <mergeCell ref="I15:N15"/>
     <mergeCell ref="R9:R12"/>
+    <mergeCell ref="I29:P29"/>
+    <mergeCell ref="F40:H40"/>
     <mergeCell ref="F15:H15"/>
+    <mergeCell ref="I31:P31"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F34:H34"/>
     <mergeCell ref="F8:R8"/>
     <mergeCell ref="F2:R2"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="Q33:R33"/>
+    <mergeCell ref="I32:P32"/>
     <mergeCell ref="O18:R18"/>
     <mergeCell ref="Q9:Q12"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="O42:R42"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="F33:H33"/>
     <mergeCell ref="P9:P12"/>
     <mergeCell ref="M6:R6"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="F39:H39"/>
+    <mergeCell ref="Q35:R35"/>
     <mergeCell ref="B14:E14"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="S30:T30"/>
+    <mergeCell ref="I38:P38"/>
+    <mergeCell ref="I40:P40"/>
     <mergeCell ref="E9:F12"/>
+    <mergeCell ref="O43:T43"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="Q31:R31"/>
     <mergeCell ref="B15:E15"/>
+    <mergeCell ref="I41:P41"/>
     <mergeCell ref="E13:F13"/>
+    <mergeCell ref="F37:H37"/>
+    <mergeCell ref="Q32:R32"/>
+    <mergeCell ref="S32:T32"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B30:E30"/>
     <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B27:T27"/>
     <mergeCell ref="F6:J6"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="I37:P37"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="S35:T35"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="N25:O25"/>
     <mergeCell ref="I18:N18"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="F24:M24"/>
     <mergeCell ref="P3:R3"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="B45:F45"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="K6:L6"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="Q28:R28"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="I42:N42"/>
     <mergeCell ref="B7:E7"/>
+    <mergeCell ref="I44:N44"/>
+    <mergeCell ref="I33:P33"/>
     <mergeCell ref="F16:H16"/>
     <mergeCell ref="K7:L7"/>
+    <mergeCell ref="I35:P35"/>
+    <mergeCell ref="O22:R22"/>
     <mergeCell ref="B9:D12"/>
+    <mergeCell ref="I30:P30"/>
+    <mergeCell ref="P25:T25"/>
+    <mergeCell ref="O44:T44"/>
     <mergeCell ref="I13:O13"/>
+    <mergeCell ref="B20:E22"/>
     <mergeCell ref="F4:H4"/>
+    <mergeCell ref="G45:H45"/>
     <mergeCell ref="B8:E8"/>
+    <mergeCell ref="I45:N45"/>
     <mergeCell ref="C13:D13"/>
+    <mergeCell ref="G46:H46"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>

</xml_diff>